<commit_message>
Update comparison logic in `comparison_diff_gpt.py` to enforce strict rules for indicator consolidation; binary file `comparison.xlsx` updated.
</commit_message>
<xml_diff>
--- a/outputs/resultats/td/2025_t2_vs_2025_t1/text_comparison.xlsx
+++ b/outputs/resultats/td/2025_t2_vs_2025_t1/text_comparison.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analyse complète" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Analyse complète'!$A$1:$J$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Analyse complète'!$A$1:$J$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -466,17 +466,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J24"/>
+  <dimension ref="A1:J26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
     <col width="35" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="70" customWidth="1" min="6" max="6"/>
     <col width="70" customWidth="1" min="7" max="7"/>
-    <col width="70" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
     <col width="70" customWidth="1" min="9" max="9"/>
     <col width="25" customWidth="1" min="10" max="10"/>
   </cols>
@@ -484,42 +484,42 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Titre</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Sous-section</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Page T1</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Page T2</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Type de changement</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Texte exact T1</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Texte exact T2</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Nouvelle idée ?</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Sous-section</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Titre</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Page T1</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Page T2</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Type de changement</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Texte exact T1</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Texte exact T2</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
@@ -536,36 +536,40 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>Gestion des risques</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Facteurs de risque qui pourraient avoir une incidence sur les résultats futurs</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Ajout</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Outre les risques décrits dans la section « Gestion des risques » du rapport de gestion de 2024 de la Banque et du présent document, divers autres facteurs de risque, dont bon nombre échappent au contrôle de la Banque et dont les effets peuvent être difficiles à prévoir, pourraient faire en sorte que les résultats de la Banque diffèrent de façon importante des prévisions, objectifs et estimations de la Banque, ou pourraient nuire à la réputation de la Banque ou compromettre la viabilité de son modèle d'affaires. Tous les énoncés prospectifs, y compris les énoncés prospectifs inclus dans le présent rapport de gestion, sont naturellement assujettis à des risques inhérents et à des incertitudes, de nature générale et spécifique, qui peuvent faire en sorte que les résultats réels de la Banque diffèrent considérablement de ceux avancés dans les prévisions, les objectifs, les estimations et les énoncés prospectifs. Certains de ces facteurs sont présentés dans la section « Facteurs de risque et gestion des risques » du rapport de gestion de 2024 et dans la section « Gestion des risques » du présent document, et d'autres sont cités dans la section « Mise en garde à l'égard des énoncés prospectifs » du présent document. La Banque a mis à jour les facteurs de risque suivants pour tenir compte des changements dans l'environnement externe.</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
           <t>Oui</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Facteurs de risque qui pourraient avoir une incidence sur les résultats futurs</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Gestion des risques</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="2" t="inlineStr"/>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Ajout</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Outre les risques décrits dans la section « Gestion des risques » du rapport de gestion de 2024 de la Banque et du présent document, divers autres facteurs de risque, dont bon nombre échappent au contrôle de la Banque et dont les effets peuvent être difficiles à prévoir, pourraient faire en sorte que les résultats de la Banque diffèrent de façon importante des prévisions, objectifs et estimations de la Banque, ou pourraient nuire à la réputation de la Banque ou compromettre la viabilité de son modèle d'affaires. Tous les énoncés prospectifs, y compris les énoncés prospectifs inclus dans le présent rapport de gestion, sont naturellement assujettis à des risques inhérents et à des incertitudes, de nature générale et spécifique, qui peuvent faire en sorte que les résultats réels de la Banque diffèrent considérablement de ceux avancés dans les prévisions, les objectifs, les estimations et les énoncés prospectifs. Certains de ces facteurs sont présentés dans la section « Facteurs de risque et gestion des risques » du rapport de gestion de 2024 et dans la section « Gestion des risques » du présent document, et d'autres sont cités dans la section « Mise en garde à l'égard des énoncés prospectifs » du présent document. La Banque a mis à jour les facteurs de risque suivants pour tenir compte des changements dans l'environnement externe.</t>
-        </is>
-      </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Une nouvelle sous section sur les facteurs de risque a été ajoutée, soulignant des risques potentiels qui pourraient affecter les résultats futurs de la banque. Ce changement est substantiel car il introduit de nouveaux éléments de risque qui nécessitent une attention accrue. Cela implique une escalade pour évaluer l'impact de ces risques sur la stratégie globale de la banque
-L'ajout de nouveaux facteurs de risque pourrait influencer la perception du marché et la stratégie de gestion des risques de la banque</t>
+          <t>Une nouvelle sous section sur les facteurs de risque a été ajoutée, soulignant des risques potentiels qui pourraient affecter les résultats futurs de la banque. Ce changement est substantiel car il introduit de nouveaux éléments de risque qui nécessitent une attention particulière. Cela implique que la banque doit évaluer ces risques et ajuster ses stratégies de gestion des risques en conséquence
+L'ajout de nouveaux facteurs de risque pourrait indiquer une exposition accrue à des incertitudes externes, nécessitant une surveillance renforcée</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr"/>
@@ -573,36 +577,40 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
+          <t>Gestion des risques</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Risques géopolitiques</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr"/>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Ajout</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>En plus des risques géopolitiques présentés dans le rapport de gestion de 2024 de la Banque, l'évolution des risques géopolitiques et des risques liés aux politiques, au commerce et à l'impôt, notamment l'application de nouveaux tarifs douaniers ou de tarifs douaniers plus élevés sur les marchandises importées aux États-Unis ou la menace de le faire et l'imposition de tarifs de représailles ainsi que l'adoption des dispositions législatives de nature fiscale récemment proposées aux États-Unis, peut amplifier l'incertitude économique et la volatilité des marchés, perturber les chaînes d'approvisionnement et les activités commerciales à l'échelle mondiale, ébranler la confiance des entreprises ou entraîner d'autres conséquences défavorables. Par exemple, les tarifs douaniers risquent de faire hausser les prix et baisser la demande des marchandises importées, pesant sur les activités des pays importateurs et exportateurs. L'imposition de tarifs douaniers très élevés pourrait couper court aux activités commerciales et entraîner des pénuries dans l'ensemble de la chaîne d'approvisionnement. Bien que la nature et l'ampleur des risques puissent varier, ils ont le potentiel de perturber la croissance économique, d'accroître la volatilité des marchés des capitaux, ce qui pourrait avoir une incidence sur la situation financière et les activités de négociation et autres que de négociation de la Banque, d'agir sur la liquidité des marchés et les coûts de financement, d'exercer des pressions sur les conditions de crédit et d'influencer directement et indirectement la conjoncture économique et commerciale et certains secteurs de sorte que la Banque et ses clients pourraient en souffrir. Pour de plus amples renseignements sur les perspectives économiques, se reporter à la rubrique « Sommaire et perspectives économiques » du présent document.</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
           <t>Oui</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Risques géopolitiques</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Gestion des risques</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="2" t="inlineStr"/>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Ajout</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>En plus des risques géopolitiques présentés dans le rapport de gestion de 2024 de la Banque, l'évolution des risques géopolitiques et des risques liés aux politiques, au commerce et à l'impôt, notamment l'application de nouveaux tarifs douaniers ou de tarifs douaniers plus élevés sur les marchandises importées aux États-Unis ou la menace de le faire et l'imposition de tarifs de représailles ainsi que l'adoption des dispositions législatives de nature fiscale récemment proposées aux États-Unis, peut amplifier l'incertitude économique et la volatilité des marchés, perturber les chaînes d'approvisionnement et les activités commerciales à l'échelle mondiale, ébranler la confiance des entreprises ou entraîner d'autres conséquences défavorables. Par exemple, les tarifs douaniers risquent de faire hausser les prix et baisser la demande des marchandises importées, pesant sur les activités des pays importateurs et exportateurs. L'imposition de tarifs douaniers très élevés pourrait couper court aux activités commerciales et entraîner des pénuries dans l'ensemble de la chaîne d'approvisionnement. Bien que la nature et l'ampleur des risques puissent varier, ils ont le potentiel de perturber la croissance économique, d'accroître la volatilité des marchés des capitaux, ce qui pourrait avoir une incidence sur la situation financière et les activités de négociation et autres que de négociation de la Banque, d'agir sur la liquidité des marchés et les coûts de financement, d'exercer des pressions sur les conditions de crédit et d'influencer directement et indirectement la conjoncture économique et commerciale et certains secteurs de sorte que la Banque et ses clients pourraient en souffrir. Pour de plus amples renseignements sur les perspectives économiques, se reporter à la rubrique « Sommaire et perspectives économiques » du présent document.</t>
-        </is>
-      </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Une nouvelle sous section sur les risques géopolitiques a été ajoutée, détaillant les impacts potentiels des politiques commerciales et fiscales. Ce changement est substantiel car il introduit des risques externes significatifs qui pourraient affecter la banque. Cela implique une escalade pour évaluer comment ces risques pourraient influencer les opérations et la stratégie de la banque
-Les risques géopolitiques peuvent entraîner une volatilité accrue et affecter les opérations internationales de la banque</t>
+          <t>Une nouvelle sous section sur les risques géopolitiques a été ajoutée, détaillant les impacts potentiels des tensions commerciales et politiques. Ce changement est substantiel car il met en lumière des risques externes qui pourraient affecter la banque. Cela implique que la banque doit surveiller ces développements et ajuster ses stratégies en conséquence
+Les risques géopolitiques peuvent entraîner une volatilité accrue des marchés et affecter la stabilité financière de la banque</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr"/>
@@ -610,7 +618,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Oui</t>
+          <t>Gestion des risques</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -618,20 +626,19 @@
           <t>Surveillance réglementaire et risque de conformité</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Gestion des risques</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Ajout</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr"/>
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>En plus des risques décrits à la rubrique « Surveillance réglementaire et conformité » du rapport de gestion de 2024 de la Banque, les organismes de réglementation ont indiqué la possibilité d'intensifier les conséquences pour les banques qui ne résolvent pas en temps opportun les problèmes en cours ou qui ont des problèmes à répétition. Un retard quant au respect d'une exigence réglementaire risquerait également d'entraver les progrès de la Banque à l'égard d'autres exigences. L'incapacité de répondre en temps opportun aux exigences réglementaires, y compris l'obligation de mettre en œuvre un programme de gestion de la conformité conformément aux normes réglementaires, pourrait mener à l'imposition d'amendes, de pénalités, de restrictions commerciales, de limites
 liées aux distributions de capital par les filiales ou de mesures coercitives supplémentaires, à l'accroissement des obligations en matière de fonds propres ou de liquidité, à une surveillance réglementaire accrue et à d'autres conséquences négatives pouvant s'avérer importantes.
@@ -657,10 +664,15 @@
 Les fonds propres exposés au risque de marché sont calculés selon l'approche standard de Bâle III. La Banque continue d'utiliser la valeur à risque (VaR) comme mesure de gestion interne pour surveiller et contrôler le risque de marché.</t>
         </is>
       </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Une nouvelle sous section sur la surveillance réglementaire et le risque de conformité a été ajoutée, indiquant des conséquences potentielles pour la non conformité. Ce changement est substantiel car il met en lumière des risques de conformité accrus qui pourraient avoir des impacts significatifs. Cela implique une escalade pour s'assurer que la banque est préparée à répondre à ces des exigences prudentielles
-Les nouvelles exigences de conformité peuvent entraîner des coûts supplémentaires et affecter la réputation de la banque</t>
+          <t>Une nouvelle sous section sur la surveillance réglementaire et le risque de conformité a été ajoutée, soulignant les conséquences potentielles d'une non conformité. Ce changement est substantiel car il met en évidence des risques de conformité qui pourraient avoir des impacts significatifs. Cela implique que la banque doit renforcer ses contrôles de conformité pour éviter des sanctions potentielles
+Les risques de non conformité peuvent entraîner des amendes et nuire à la réputation de la banque, affectant sa stabilité à long terme</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr"/>
@@ -668,36 +680,40 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
+          <t>Gestion du capital</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Exigences en matière de fonds propres du BSIF en vertu de Bâle III</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr"/>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Ajout</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr"/>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Au 30 avril 2025, le ratio des fonds propres de catégorie 1 sous forme d'actions ordinaires, le ratio des fonds propres de catégorie 1 et le ratio du total des fonds propres de la Banque étaient respectivement de 14,9 %, 16,6 %, et 18,5 %. Le ratio des fonds propres de catégorie 1 sous forme d'actions ordinaires de la Banque a augmenté par rapport au ratio de 13,1 % au 31 octobre 2024, ce qui est principalement attribuable à la vente des actions de Schwab et à la génération interne de capitaux, contrebalancées par le rachat d'actions ordinaires aux fins d'annulation, la croissance des actifs pondérés en fonction des risques dans plusieurs secteurs et l'incidence de la restructuration du bilan aux États-Unis.</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
           <t>Oui</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Exigences en matière de fonds propres du BSIF en vertu de Bâle III</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Gestion du capital</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Ajout</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>Au 30 avril 2025, le ratio des fonds propres de catégorie 1 sous forme d'actions ordinaires, le ratio des fonds propres de catégorie 1 et le ratio du total des fonds propres de la Banque étaient respectivement de 14,9 %, 16,6 %, et 18,5 %. Le ratio des fonds propres de catégorie 1 sous forme d'actions ordinaires de la Banque a augmenté par rapport au ratio de 13,1 % au 31 octobre 2024, ce qui est principalement attribuable à la vente des actions de Schwab et à la génération interne de capitaux, contrebalancées par le rachat d'actions ordinaires aux fins d'annulation, la croissance des actifs pondérés en fonction des risques dans plusieurs secteurs et l'incidence de la restructuration du bilan aux États-Unis.</t>
-        </is>
-      </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Les ratios de fonds propres de la Banque au avril ont été ajoutés, montrant une augmentation par rapport à octobre. Ce changement est substantiel car il indique une amélioration de la position de capital, influencée par des transactions stratégiques et la gestion du bilan. Cela nécessite une confirmation pour s'assurer que ces niveaux sont maintenus et conformes aux des exigences prudentielles
-Renforcement de la position de capital de la banque</t>
+          <t>Les ratios de fonds propres de la Banque ont été mis à jour pour avril, montrant une augmentation par rapport à octobre. Ce changement est substantiel car il reflète une amélioration de la position de capital de la Banque, influencée par des transactions stratégiques et des ajustements internes. Cela implique une surveillance continue pour s'assurer que ces niveaux de capital sont maintenus ou améliorés
+Amélioration de la position de capital de la Banque, renforçant sa capacité à absorber les pertes</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr"/>
@@ -705,142 +721,116 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
+          <t>Gestion du capital</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Exigences en matière de fonds propres du BSIF en vertu de Bâle III</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr"/>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Ajout</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr"/>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Au 30 avril 2025, le ratio de levier de la Banque était de 4,7 %. Le ratio de levier de la Banque a augmenté par rapport au ratio de 4,2 % au 31 octobre 2024, ce qui est principalement attribuable à la vente des actions de Schwab et à la génération interne de capitaux, contrebalancées par le rachat d'actions ordinaires aux fins d'annulation, l'augmentation de l'exposition dans plusieurs secteurs et l'incidence de la restructuration du bilan aux États-Unis.</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
           <t>Oui</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Le ratio de levier de la Banque a augmenté à en avril, par rapport à en octobre. Ce changement est substantiel car il indique une amélioration de la capacité de la Banque à gérer ses actifs et passifs, influencée par des transactions stratégiques. Cela nécessite une surveillance pour s'assurer que le ratio de levier reste dans les limites réglementaires
+Augmentation du ratio de levier, améliorant la capacité de la Banque à gérer ses actifs et passifs</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Gestion du capital</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Exigences en matière de fonds propres du BSIF en vertu de Bâle III</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Gestion du capital</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Ajout</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>Au 30 avril 2025, le ratio de levier de la Banque était de 4,7 %. Le ratio de levier de la Banque a augmenté par rapport au ratio de 4,2 % au 31 octobre 2024, ce qui est principalement attribuable à la vente des actions de Schwab et à la génération interne de capitaux, contrebalancées par le rachat d'actions ordinaires aux fins d'annulation, l'augmentation de l'exposition dans plusieurs secteurs et l'incidence de la restructuration du bilan aux États-Unis.</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>Le ratio de levier de la Banque a augmenté à au avril, par rapport à en octobre. Ce changement est substantiel car il reflète une amélioration de la capacité de la banque à absorber les pertes, influencée par des transactions stratégiques. Cela nécessite une confirmation pour garantir que cette amélioration est durable et conforme aux normes prudentielles
-Amélioration de la capacité d'absorption des pertes de la banque</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Exigences en matière de fonds propres du BSIF en vertu de Bâle III</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Gestion du capital</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>Ajout</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>Le tableau ci-après présente des détails sur la situation des fonds propres réglementaires de la Banque.</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>Un tableau détaillant la situation des fonds propres réglementaires de la Banque a été ajouté. Ce changement est substantiel car il fournit une vue d'ensemble des niveaux de capital, essentielle pour évaluer la santé financière de la banque. Cela implique de s'assurer que ces informations sont correctement intégrées dans les rapports de surveillance
-Amélioration de la transparence sur la situation des fonds propres</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr"/>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Modification</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Le 1 er février 2023, le BSIF a mis en œuvre les règles de fonds propres révisées qui tiennent compte des réformes de Bâle III et de certains ajustements afin de les adapter à leur mise en œuvre au Canada. Ces règles révisées comprennent des modifications aux exigences à l'égard du calcul du risque de crédit et du risque opérationnel ainsi que des modifications de la ligne directrice Exigences de levier pour inclure une exigence selon laquelle les banques d'importance systémique intérieure (BISI) doivent maintenir un coussin de ratio de levier de 0,50 % en plus de l'exigence réglementaire minimale de 3,0 %. Ce coussin s'applique également au ratio de levier TLAC. Le 1 er novembre 2023, le BSIF a mis en œuvre la deuxième et dernière phase des réformes de Bâle III relatives au calcul des actifs pondérés en fonction des risques au titre du risque lié au rajustement de la valeur de crédit (RVC) et au titre du risque de marché. De plus, à compter du 1 er novembre 2023, le plancher réglementaire des fonds propres est passé de 65 % des actifs pondérés en fonction des risques pour l'exercice 2023 à 67,5 % des actifs pondérés en fonction des risques pour l'exercice 2024.</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Le BSIF a mis en œuvre les réformes de Bâle III et certains ajustements afin de les adapter à leur mise en œuvre au Canada. Ces réformes ont une incidence sur le calcul du risque de crédit, du risque de marché et du risque opérationnel pour les banques canadiennes, et modifient la ligne directrice Exigences de levier pour inclure une exigence selon laquelle les banques d'importance systémique intérieure (BISI) doivent maintenir un coussin de ratio de levier de 0,50 % en plus de l'exigence réglementaire minimale de 3,0 %. Ce coussin s'applique également au ratio de levier TLAC.</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>Les détails sur la mise en œuvre des réformes de en février et novembre ont été supprimés, affectant le calcul des actifs pondérés en fonction des risques. Ce changement est substantiel car il modifie la compréhension des exigences de fonds propres et de levier pour les banques canadiennes. Cela nécessite une réévaluation des stratégies de gestion des risques et de capital pour s'assurer de la conformité continue
+Modification des exigences de fonds propres et de levier, impactant potentiellement la stratégie de capital des banques</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Gestion du capital</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Exigences en matière de fonds propres du BSIF en vertu de Bâle III</t>
+          <t>Informations communiquées par les banques d'importance systémique mondiale</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Gestion du capital</t>
+          <t>34</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr"/>
-      <c r="E8" s="3" t="inlineStr"/>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Suppression</t>
+        </is>
+      </c>
       <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>Modification</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>Le 1 er février 2023, le BSIF a mis en œuvre les règles de fonds propres révisées qui tiennent compte des réformes de Bâle III et de certains ajustements afin de les adapter à leur mise en œuvre au Canada. Ces règles révisées comprennent des modifications aux exigences à l'égard du calcul du risque de crédit et du risque opérationnel ainsi que des modifications de la ligne directrice Exigences de levier pour inclure une exigence selon laquelle les banques d'importance systémique intérieure (BISI) doivent maintenir un coussin de ratio de levier de 0,50 % en plus de l'exigence réglementaire minimale de 3,0 %. Ce coussin s'applique également au ratio de levier TLAC. Le 1 er novembre 2023, le BSIF a mis en œuvre la deuxième et dernière phase des réformes de Bâle III relatives au calcul des actifs pondérés en fonction des risques au titre du risque lié au rajustement de la valeur de crédit (RVC) et au titre du risque de marché. De plus, à compter du 1 er novembre 2023, le plancher réglementaire des fonds propres est passé de 65 % des actifs pondérés en fonction des risques pour l'exercice 2023 à 67,5 % des actifs pondérés en fonction des risques pour l'exercice 2024.</t>
-        </is>
-      </c>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>Le BSIF a mis en œuvre les réformes de Bâle III et certains ajustements afin de les adapter à leur mise en œuvre au Canada. Ces réformes ont une incidence sur le calcul du risque de crédit, du risque de marché et du risque opérationnel pour les banques canadiennes, et modifient la ligne directrice Exigences de levier pour inclure une exigence selon laquelle les banques d'importance systémique intérieure (BISI) doivent maintenir un coussin de ratio de levier de 0,50 % en plus de l'exigence réglementaire minimale de 3,0 %. Ce coussin s'applique également au ratio de levier TLAC.</t>
-        </is>
-      </c>
-      <c r="I8" s="3" t="inlineStr">
-        <is>
-          <t>Les détails sur la mise en œuvre des réformes de et le plancher réglementaire des fonds propres ont été supprimés. Ce changement est substantiel car il omet des informations cruciales sur les exigences de fonds propres et les ajustements réglementaires. Cela nécessite une escalade pour clarifier l'impact de ces réformes sur la stabilité financière de la banque
-Potentiel impact sur la conformité réglementaire et la gestion des fonds propres</t>
-        </is>
-      </c>
-      <c r="J8" s="3" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>Informations communiquées par les banques d'importance systémique mondiale</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>Gestion du capital</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr"/>
-      <c r="E9" s="3" t="inlineStr"/>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>Suppression</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>Le Conseil de stabilité financière (CSF), après consultation avec le CBCB et les instances nationales, désigne les BISM. La méthodologie d'évaluation des BISM s'appuie sur les renseignements fournis par les plus grandes banques internationales. Treize indicateurs sont utilisés dans la méthodologie d'évaluation des BISM pour mesurer l'importance systémique. Le score pour un indicateur particulier est obtenu en divisant la valeur fournie par la banque considérée par le montant total fourni par les banques de l'échantillon pour cet indicateur inclus dans l'évaluation. Par conséquent, le score pour un indicateur de la banque considérée dépend des résultats et des renseignements fournis par les autres banques d'envergure internationale.
 La Banque doit publier les treize indicateurs utilisés dans le cadre d'évaluation fondé sur des indicateurs des BISM. La communication publique des données de fin d'exercice est requise chaque année, au plus tard à la date de la communication publique des données financières du premier trimestre de l'exercice suivant de la banque à l'intention des actionnaires.
@@ -854,80 +844,43 @@
 Au 31 janvier 2025, le ratio de levier de la Banque était de 4,2 %. Le ratio de levier de la Banque est demeuré relativement stable par rapport au ratio de 4,2 % au 31 octobre 2024, ce qui est principalement attribuable à la génération interne de capitaux, contrebalancée par l'augmentation de l'exposition dans plusieurs secteurs et l'incidence de la restructuration du bilan aux États-Unis.</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr"/>
-      <c r="I9" s="3" t="inlineStr">
-        <is>
-          <t>Une sous section entière concernant les banques d'importance systémique mondiale a été supprimée. Ce changement est substantiel car il retire des informations critiques sur les obligations de divulgation et les exigences de fonds propres supplémentaires. Cela nécessite une escalade pour évaluer l'impact de cette suppression sur la conformité réglementaire de la banque
-Risque de non conformité aux exigences de divulgation pour les banques systémiques</t>
-        </is>
-      </c>
-      <c r="J9" s="3" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>Calcul de la VaR</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr"/>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>La section sur les banques d'importance systémique mondiale a été supprimée, y compris les détails sur les exigences de fonds propres supplémentaires. Ce changement est substantiel car il affecte la transparence et la compréhension des obligations réglementaires de la Banque. Cela nécessite une escalade pour clarifier les implications de cette suppression sur la conformité réglementaire
+Suppression d'informations critiques sur les obligations réglementaires des banques d'importance systémique</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Gestion des risques</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr"/>
-      <c r="E10" s="4" t="inlineStr"/>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>Modification</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>La VaR moyenne a diminué d'un trimestre à l'autre en raison des variations des positions dans des titres à revenu fixe et du resserrement des écarts de taux.</t>
-        </is>
-      </c>
-      <c r="H10" s="4" t="inlineStr">
-        <is>
-          <t>La VaR moyenne a augmenté par rapport à celle du trimestre précédent en raison de la volatilité des marchés ayant influé sur certains facteurs de risque, notamment les écarts de taux et les marchandises.</t>
-        </is>
-      </c>
-      <c r="I10" s="4" t="inlineStr">
-        <is>
-          <t>La tendance de la mesure de risque de marché moyenne a changé de diminution à augmentation entre les trimestres. Ce changement est substantiel car il reflète une modification de l'exposition au risque de marché de la banque. Cela implique que la banque doit ajuster ses stratégies de gestion du risque pour s'adapter à la nouvelle volatilité du marché
-L'augmentation de la mesure de risque de marché moyenne indique une exposition accrue aux fluctuations du marché, nécessitant une réévaluation des stratégies de couverture</t>
-        </is>
-      </c>
-      <c r="J10" s="4" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>intro</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>Gestion des risques</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr"/>
-      <c r="E11" s="4" t="inlineStr"/>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr"/>
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>Suppression</t>
         </is>
       </c>
-      <c r="G11" s="4" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>Faire croître la rentabilité des résultats financiers en comptant sur l'équilibre entre les produits, les charges et la croissance des fonds propres implique de prendre des risques mesurés et de les gérer en tenant compte de l'appétit de la Banque pour le risque. L'objectif de la Banque est d'obtenir un rendement stable et durable pour chaque dollar de risque qu'elle prend, tout en accordant une grande importance à l'investissement dans ses entreprises afin d'atteindre ses objectifs stratégiques futurs.
 Les entreprises et les activités de la Banque sont exposées à un grand nombre de risques qui ont été recensés et définis dans le cadre de gestion des risques à l'échelle de l'entreprise. La tolérance de la Banque à ces risques est définie dans la prise de position sur l'« Appétit pour le risque de l'entreprise », élaborée
@@ -942,11 +895,114 @@
 Les fonds propres exposés au risque de marché sont calculés selon l'approche standard. La Banque continue d'utiliser la valeur à risque (VaR) comme mesure de gestion interne pour surveiller et contrôler le risque de marché.</t>
         </is>
       </c>
-      <c r="H11" s="4" t="inlineStr"/>
+      <c r="G9" s="3" t="inlineStr"/>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>La section sur la gestion des risques a été entièrement supprimée entre le premier et le deuxième trimestre. Ce changement est substantiel car il retire des informations cruciales sur la manière dont la banque gère et perçoit ses risques. Cela implique une nécessité urgente de comprendre pourquoi cette information a été retirée et d'évaluer les impacts potentiels sur la surveillance des risques de la banque
+La suppression de cette section pourrait indiquer un changement significatif dans la stratégie de gestion des risques de la banque, ce qui pourrait affecter sa stabilité financière</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Gestion des risques</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Calcul de la VaR</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Modification</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>La VaR moyenne a diminué d'un trimestre à l'autre en raison des variations des positions dans des titres à revenu fixe et du resserrement des écarts de taux.</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>La VaR moyenne a augmenté par rapport à celle du trimestre précédent en raison de la volatilité des marchés ayant influé sur certains facteurs de risque, notamment les écarts de taux et les marchandises.</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>La tendance de la mesure de risque de marché moyenne a changé de diminution à augmentation entre les trimestres. Ce changement est substantiel car il reflète une augmentation de la volatilité des marchés, influençant les facteurs de risque. Cela implique que la banque doit ajuster ses stratégies de gestion des risques pour s'adapter à cette nouvelle volatilité
+L'augmentation de la mesure de risque de marché moyenne pourrait indiquer une exposition accrue aux fluctuations du marché, nécessitant une surveillance renforcée</t>
+        </is>
+      </c>
+      <c r="J10" s="4" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Gestion des risques</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Risque de taux d'intérêt (autre que de négociation) structurel</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Modification</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Au 31 janvier 2025, une augmentation immédiate et soutenue de 100 pdb des taux d'intérêt aurait eu une incidence négative de 2 573 millions de dollars sur la valeur économique des capitaux propres attribuables aux actionnaires de la Banque, soit une augmentation de 84 millions de dollars par rapport à celle du trimestre précédent, et une incidence positive de 597 millions de dollars sur les produits d'intérêts nets de la Banque, soit une diminution de 123 millions de dollars par rapport à celle du trimestre précédent. Une diminution immédiate et soutenue de 100 pdb des taux d'intérêt aurait eu une incidence positive de 2 056 millions de dollars sur la valeur économique des capitaux propres attribuables aux actionnaires de la Banque, soit une augmentation de 142 millions de dollars par rapport à celle du trimestre précédent, et une incidence négative de 789 millions de dollars sur les produits d'intérêts nets de la Banque, soit une diminution de 194 millions de dollars par rapport à celle du trimestre précédent. L'augmentation d'un trimestre à l'autre de la sensibilité de la valeur économique des capitaux propres attribuables aux actionnaires découle en partie de la conversion des monnaies étrangères ainsi que d'une légère augmentation des actifs nets à taux fixe détenus. La diminution d'un trimestre à l'autre de la sensibilité des produits d'intérêts nets est principalement attribuable à la mise en œuvre d'autres stratégies de couverture au cours du trimestre.</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>Au 30 avril 2025, une augmentation immédiate et soutenue de 100 pdb des taux d'intérêt aurait eu une incidence négative de 2 612 millions de dollars sur la valeur économique des capitaux propres attribuables aux actionnaires de la Banque, soit une augmentation de 39 millions de dollars par rapport à celle du trimestre précédent, et une incidence positive de 679 millions de dollars sur les produits d'intérêts nets de la Banque, soit une augmentation de 82 millions de dollars par rapport à celle du trimestre précédent. Une diminution immédiate et soutenue de 100 pdb des taux d'intérêt aurait eu une incidence positive de 2 116 millions de dollars sur la valeur économique des capitaux propres attribuables aux actionnaires de la Banque, soit une augmentation de 60 millions de dollars par rapport à celle du trimestre précédent, et une incidence négative de 769 millions de dollars sur les produits d'intérêts nets de la Banque, soit une diminution de 20 millions de dollars par rapport à celle du trimestre précédent. L'augmentation d'un trimestre à l'autre de la sensibilité de la valeur économique des capitaux propres attribuables aux actionnaires découle d'une légère hausse des actifs à taux fixe détenus tandis que la sensibilité des produits d'intérêts nets est demeurée relativement stable au cours du trimestre considéré.</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>La section sur la gestion des risques a été entièrement supprimée entre le premier et le deuxième trimestre. Ce changement est substantiel car il retire des informations cruciales sur la manière dont la banque gère et perçoit ses risques. Cela implique une nécessité de vérifier si cette suppression est intentionnelle et si les informations ont été déplacées ou remplacées ailleurs
-La suppression de cette section pourrait indiquer un changement dans la stratégie de gestion des risques ou une omission involontaire, ce qui nécessite une attention particulière</t>
+          <t>Les chiffres concernant l'impact des variations des taux d'intérêt sur la valeur économique des capitaux propres et les produits d'intérêts nets ont été mis à jour. Ce changement est substantiel car il reflète une modification des sensibilités financières de la banque. Cela implique que la banque doit confirmer ces chiffres pour s'assurer qu'ils reflètent correctement sa position actuelle
+Les nouvelles données indiquent une sensibilité accrue aux variations des taux d'intérêt, ce qui pourrait affecter la rentabilité future</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr"/>
@@ -954,40 +1010,48 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Gestion des risques</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Risque de taux d'intérêt (autre que de négociation) structurel</t>
+          <t>Actifs liquides</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Gestion des risques</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="inlineStr"/>
-      <c r="E12" s="4" t="inlineStr"/>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Modification</t>
+        </is>
+      </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Modification</t>
+          <t>Le NSFR de la Banque pour le trimestre clos le 31 janvier 2025 a été de 116 % (116 % pour le trimestre clos le 31 octobre 2024), correspondant à un montant excédentaire de 158 milliards de dollars, ce qui respecte les exigences réglementaires. Le ratio est demeuré stable, la hausse des dépôts ayant été contrebalancée par la croissance des actifs.</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>Au 31 janvier 2025, une augmentation immédiate et soutenue de 100 pdb des taux d'intérêt aurait eu une incidence négative de 2 573 millions de dollars sur la valeur économique des capitaux propres attribuables aux actionnaires de la Banque, soit une augmentation de 84 millions de dollars par rapport à celle du trimestre précédent, et une incidence positive de 597 millions de dollars sur les produits d'intérêts nets de la Banque, soit une diminution de 123 millions de dollars par rapport à celle du trimestre précédent. Une diminution immédiate et soutenue de 100 pdb des taux d'intérêt aurait eu une incidence positive de 2 056 millions de dollars sur la valeur économique des capitaux propres attribuables aux actionnaires de la Banque, soit une augmentation de 142 millions de dollars par rapport à celle du trimestre précédent, et une incidence négative de 789 millions de dollars sur les produits d'intérêts nets de la Banque, soit une diminution de 194 millions de dollars par rapport à celle du trimestre précédent. L'augmentation d'un trimestre à l'autre de la sensibilité de la valeur économique des capitaux propres attribuables aux actionnaires découle en partie de la conversion des monnaies étrangères ainsi que d'une légère augmentation des actifs nets à taux fixe détenus. La diminution d'un trimestre à l'autre de la sensibilité des produits d'intérêts nets est principalement attribuable à la mise en œuvre d'autres stratégies de couverture au cours du trimestre.</t>
+          <t>Le NSFR de la Banque au 30 avril 2025 était de 119 % (116 % au 31 octobre 2024), correspondant à un montant excédentaire de 183 milliards de dollars, ce qui respecte les exigences réglementaires. L'augmentation du NSFR est principalement attribuable au produit tiré de la vente de la participation en actions dans Schwab.</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>Au 30 avril 2025, une augmentation immédiate et soutenue de 100 pdb des taux d'intérêt aurait eu une incidence négative de 2 612 millions de dollars sur la valeur économique des capitaux propres attribuables aux actionnaires de la Banque, soit une augmentation de 39 millions de dollars par rapport à celle du trimestre précédent, et une incidence positive de 679 millions de dollars sur les produits d'intérêts nets de la Banque, soit une augmentation de 82 millions de dollars par rapport à celle du trimestre précédent. Une diminution immédiate et soutenue de 100 pdb des taux d'intérêt aurait eu une incidence positive de 2 116 millions de dollars sur la valeur économique des capitaux propres attribuables aux actionnaires de la Banque, soit une augmentation de 60 millions de dollars par rapport à celle du trimestre précédent, et une incidence négative de 769 millions de dollars sur les produits d'intérêts nets de la Banque, soit une diminution de 20 millions de dollars par rapport à celle du trimestre précédent. L'augmentation d'un trimestre à l'autre de la sensibilité de la valeur économique des capitaux propres attribuables aux actionnaires découle d'une légère hausse des actifs à taux fixe détenus tandis que la sensibilité des produits d'intérêts nets est demeurée relativement stable au cours du trimestre considéré.</t>
+          <t>Non</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>Les chiffres concernant l'impact des variations des taux d'intérêt sur la valeur économique des capitaux propres et les produits d'intérêts nets ont été mis à jour. Ce changement est substantiel car il affecte directement les projections de capital et de revenus de la banque. Cela implique que la banque doit confirmer ces chiffres pour s'assurer de leur exactitude et ajuster ses prévisions financières en conséquence
-Les nouvelles projections de sensibilité aux taux d'intérêt peuvent influencer les décisions stratégiques concernant la gestion des actifs et passifs</t>
+          <t>Le ratio de financement stable net () a augmenté, principalement en raison de la vente de la participation en actions dans Schwab. Ce changement est substantiel car il améliore la position de financement à long terme de la banque. Cela implique que la banque doit confirmer l'impact de cette vente sur sa stratégie de financement
+L'augmentation du renforce la stabilité financière de la banque, mais la dépendance à une vente unique pourrait poser des risques futurs</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr"/>
@@ -995,7 +1059,7 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Gestion des risques</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
@@ -1005,30 +1069,38 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Gestion des risques</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr"/>
-      <c r="E13" s="4" t="inlineStr"/>
+          <t>51</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Modification</t>
+        </is>
+      </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Modification</t>
+          <t>Le tableau ci-après présente la ventilation de la dette à terme de la Banque par monnaie et type de financement. Le financement à terme au 31 janvier 2025 s'élevait à 189,7 milliards de dollars (184,5 milliards de dollars au 31 octobre 2024).</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>5 Les autres actifs comprennent la participation dans Schwab, le goodwill, les autres immobilisations incorporelles, les terrains, bâtiments, matériel et mobilier, autres actifs amortissables et actifs au titre de droits d'utilisation, les actifs d'impôt différé, les montants à recevoir des courtiers et des clients et les autres actifs du bilan qui ne sont pas présentés dans les catégories ci-dessus.</t>
+          <t>Le tableau ci-après présente la ventilation de la dette à terme de la Banque par monnaie et type de financement. Le financement à terme au 30 avril 2025 s'élevait à 185,6 milliards de dollars (184,5 milliards de dollars au 31 octobre 2024).</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>5 Les autres actifs comprennent le goodwill, les autres immobilisations incorporelles, les terrains, bâtiments, matériel et mobilier, autres actifs amortissables et actifs au titre de droits d'utilisation, les actifs d'impôt différé, les montants à recevoir des courtiers et des clients et les autres actifs du bilan qui ne sont pas présentés dans les catégories ci-dessus.</t>
+          <t>Non</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>La mention de la participation dans Schwab a été supprimée de la liste des autres actifs. Ce changement est substantiel car il reflète une modification dans la composition des actifs de la banque. Cela implique de confirmer la vente ou la réévaluation de cette participation pour comprendre son impact sur le bilan
-La suppression de la participation dans Schwab indique un changement potentiel dans la structure des actifs, nécessitant une réévaluation des actifs stratégiques</t>
+          <t>Le montant du financement à terme a été mis à jour, avec une légère diminution par rapport au trimestre précédent. Ce changement est substantiel car il affecte la capacité de la banque à gérer ses obligations à long terme. Cela implique que la banque doit confirmer ces chiffres pour s'assurer qu'ils reflètent correctement sa position de financement
+La diminution du financement à terme pourrait indiquer une réduction de la capacité de la banque à lever des fonds à long terme</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr"/>
@@ -1036,7 +1108,7 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Gestion des risques</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
@@ -1046,30 +1118,38 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Gestion des risques</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="inlineStr"/>
-      <c r="E14" s="4" t="inlineStr"/>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Modification</t>
+        </is>
+      </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Modification</t>
+          <t>4 Comprennent la dette de premier rang qui est assujettie à une conversion au titre du régime de recapitalisation interne des banques. Excluent des billets structurés d'un montant de 4,0 milliards de dollars qui sont assujettis à une conversion au titre du régime de recapitalisation des banques (4,4 milliards de dollars au 31 octobre 2024).</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>Le NSFR de la Banque pour le trimestre clos le 31 janvier 2025 a été de 116 % (116 % pour le trimestre clos le 31 octobre 2024), correspondant à un montant excédentaire de 158 milliards de dollars, ce qui respecte les exigences réglementaires. Le ratio est demeuré stable, la hausse des dépôts ayant été contrebalancée par la croissance des actifs.</t>
+          <t>4 Comprennent la dette de premier rang qui est assujettie à une conversion au titre du régime de recapitalisation interne des banques. Excluent des billets structurés d'un montant de 3,7 milliards de dollars qui sont assujettis à une conversion au titre du régime de recapitalisation des banques (4,4 milliards de dollars au 31 octobre 2024).</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>Le NSFR de la Banque au 30 avril 2025 était de 119 % (116 % au 31 octobre 2024), correspondant à un montant excédentaire de 183 milliards de dollars, ce qui respecte les exigences réglementaires. L'augmentation du NSFR est principalement attribuable au produit tiré de la vente de la participation en actions dans Schwab.</t>
+          <t>Non</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>Le ratio de financement stable net a augmenté, principalement en raison de la vente de la participation en actions dans Schwab. Ce changement est substantiel car il améliore la position de financement à long terme de la banque. Cela implique de confirmer l'impact de cette vente sur la stabilité financière et de réévaluer les stratégies de financement à long terme
-L'amélioration du ratio de financement stable net renforce la capacité de la banque à maintenir ses opérations en période de stress financier</t>
+          <t>Le montant des billets structurés exclus a été réduit, ce qui affecte la composition du capital de la banque. Ce changement est substantiel car il modifie la structure de capital de la banque. Cela implique que la banque doit confirmer l'impact de cette réduction sur sa stratégie de capitalisation
+La réduction des billets structurés pourrait affecter la flexibilité financière de la banque en cas de besoin de recapitalisation</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr"/>
@@ -1077,7 +1157,7 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Gestion des risques</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
@@ -1087,30 +1167,38 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Gestion des risques</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr"/>
-      <c r="E15" s="4" t="inlineStr"/>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Modification</t>
+        </is>
+      </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>Modification</t>
+          <t>À l'exclusion des activités de négociation de prêts hypothécaires résidentiels du secteur Services bancaires de gros, la Banque a émis à l'intention d'investisseurs externes des titres adossés à des créances hypothécaires s'élevant à 1,0 milliard de dollars pour les trois mois clos le 31 janvier 2025 (0,2 milliard de dollars pour les trois mois clos le 31 janvier 2024), et les autres titres adossés à des actifs émis étaient de 0,2 milliard de dollars pour les trois mois clos le 31 janvier 2025 (néant pour les trois mois clos le 31 janvier 2024). Le montant total des billets à moyen terme non garantis et des obligations sécurisées émises pour les trois mois clos le 31 janvier 2025 était respectivement de 10,8 milliards de dollars et néant (respectivement 0,7 milliard de dollars et 4,7 milliards de dollars pour les trois mois clos le 31 janvier 2024).</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>4 Comprennent la dette de premier rang qui est assujettie à une conversion au titre du régime de recapitalisation interne des banques. Excluent des billets structurés d'un montant de 4,0 milliards de dollars qui sont assujettis à une conversion au titre du régime de recapitalisation des banques (4,4 milliards de dollars au 31 octobre 2024).</t>
+          <t>À l'exclusion des activités de négociation de prêts hypothécaires résidentiels du secteur Services bancaires de gros, la Banque a émis à l'intention d'investisseurs externes des titres adossés à des créances hypothécaires s'élevant respectivement à 1,3 milliard de dollars et 2,3 milliards de dollars pour les trois mois et six mois clos le 30 avril 2025 (respectivement 0,7 milliard de dollars et 0,8 milliard de dollars pour les trois mois et six mois clos le 30 avril 2024), et les autres titres adossés à des actifs émis étaient respectivement de néant et 0,2 milliard de dollars pour les trois mois et six mois clos le 30 avril 2025 (néant pour les trois mois et six mois clos le 30 avril 2024). La Banque a également émis des billets à moyen terme non garantis s'élevant respectivement à néant et 10,4 milliards de dollars pour les trois mois et six mois clos le 30 avril 2025 (respectivement 7,5 milliards de dollars et 8,1 milliards de dollars pour les trois mois et six mois clos le 30 avril 2024). Les obligations sécurisées émises se sont élevées à néant pour les trois mois et six mois clos le 30 avril 2025 (respectivement 10,2 milliards de dollars et 14,7 milliards de dollars pour les trois mois et six mois clos le 30 avril 2024).</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>4 Comprennent la dette de premier rang qui est assujettie à une conversion au titre du régime de recapitalisation interne des banques. Excluent des billets structurés d'un montant de 3,7 milliards de dollars qui sont assujettis à une conversion au titre du régime de recapitalisation des banques (4,4 milliards de dollars au 31 octobre 2024).</t>
+          <t>Non</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>Le montant des billets structurés exclus a été modifié. Ce changement est substantiel car il affecte le calcul des fonds propres réglementaires. Cela implique de confirmer ces chiffres pour s'assurer de leur conformité avec les des exigences prudentielles
-La modification des montants des billets structurés peut influencer la capacité de la banque à absorber les pertes en cas de crise</t>
+          <t>Les montants et les périodes pour les titres adossés à des créances hypothécaires et les billets à moyen terme non garantis ont été mis à jour. Ce changement est substantiel car il affecte la stratégie de financement de la banque. Cela implique que la banque doit confirmer ces chiffres pour s'assurer qu'ils reflètent correctement sa position de financement
+Les nouvelles émissions de titres et de billets affectent la capacité de la banque à lever des fonds sur les marchés financiers</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr"/>
@@ -1118,40 +1206,48 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Gestion du capital</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Actifs liquides</t>
+          <t>Exigences en matière de fonds propres du BSIF en vertu de Bâle III</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Gestion des risques</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr"/>
-      <c r="E16" s="4" t="inlineStr"/>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Modification</t>
+        </is>
+      </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>Modification</t>
+          <t>La réserve pour stabilité intérieure (RSI) a été augmentée pour passer de 3 % à 3,5 % au 1 er novembre 2023. La hausse de 50 pdb reflète le point de vue du BSIF quant aux mesures nécessaires pour améliorer la résilience des plus grandes banques canadiennes. La fourchette de la RSI peut actuellement s'étendre de 0 à 4 %, le niveau effectif étant modifié par le BSIF selon l'évolution du système financier canadien et de l'économie dans son ensemble.</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>À l'exclusion des activités de négociation de prêts hypothécaires résidentiels du secteur Services bancaires de gros, la Banque a émis à l'intention d'investisseurs externes des titres adossés à des créances hypothécaires s'élevant à 1,0 milliard de dollars pour les trois mois clos le 31 janvier 2025 (0,2 milliard de dollars pour les trois mois clos le 31 janvier 2024), et les autres titres adossés à des actifs émis étaient de 0,2 milliard de dollars pour les trois mois clos le 31 janvier 2025 (néant pour les trois mois clos le 31 janvier 2024). Le montant total des billets à moyen terme non garantis et des obligations sécurisées émises pour les trois mois clos le 31 janvier 2025 était respectivement de 10,8 milliards de dollars et néant (respectivement 0,7 milliard de dollars et 4,7 milliards de dollars pour les trois mois clos le 31 janvier 2024).</t>
+          <t>La réserve pour stabilité intérieure (RSI) a été augmentée pour passer de 3 % à 3,5 % au 1 er novembre 2023 et est demeurée stable depuis. La fourchette de la RSI peut actuellement s'étendre de 0 à 4 %, le niveau effectif étant modifié par le BSIF selon l'évolution du système financier canadien et de l'économie dans son ensemble.</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>À l'exclusion des activités de négociation de prêts hypothécaires résidentiels du secteur Services bancaires de gros, la Banque a émis à l'intention d'investisseurs externes des titres adossés à des créances hypothécaires s'élevant respectivement à 1,3 milliard de dollars et 2,3 milliards de dollars pour les trois mois et six mois clos le 30 avril 2025 (respectivement 0,7 milliard de dollars et 0,8 milliard de dollars pour les trois mois et six mois clos le 30 avril 2024), et les autres titres adossés à des actifs émis étaient respectivement de néant et 0,2 milliard de dollars pour les trois mois et six mois clos le 30 avril 2025 (néant pour les trois mois et six mois clos le 30 avril 2024). La Banque a également émis des billets à moyen terme non garantis s'élevant respectivement à néant et 10,4 milliards de dollars pour les trois mois et six mois clos le 30 avril 2025 (respectivement 7,5 milliards de dollars et 8,1 milliards de dollars pour les trois mois et six mois clos le 30 avril 2024). Les obligations sécurisées émises se sont élevées à néant pour les trois mois et six mois clos le 30 avril 2025 (respectivement 10,2 milliards de dollars et 14,7 milliards de dollars pour les trois mois et six mois clos le 30 avril 2024).</t>
+          <t>Non</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>Les montants et les périodes pour les titres adossés à des créances hypothécaires et les billets à moyen terme non garantis ont été mis à jour. Ce changement est substantiel car il affecte la structure de financement et la gestion des risques de crédit. Cela implique de confirmer ces chiffres pour s'assurer de leur exactitude et de leur impact sur le bilan
-Les nouvelles émissions de titres et de billets influencent la liquidité et la gestion des risques de crédit de la banque</t>
+          <t>La réserve pour stabilité intérieure (RSI) a été augmentée de à au novembre et est restée stable depuis. Ce changement est substantiel car il reflète une décision stratégique pour renforcer la résilience des grandes banques canadiennes face aux risques systémiques. Cela implique une surveillance accrue des niveaux de capital pour s'assurer que les banques maintiennent cette résilience face aux évolutions économiques
+Augmentation du niveau de capital requis pour les grandes banques, impactant leur capacité à absorber les chocs économiques</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr"/>
@@ -1159,40 +1255,48 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Gestion des risques</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Exigences en matière de fonds propres du BSIF en vertu de Bâle III</t>
+          <t>Actifs liquides</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Gestion du capital</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr"/>
-      <c r="E17" s="4" t="inlineStr"/>
+          <t>47</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Modification</t>
+        </is>
+      </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>Modification</t>
+          <t>5 Les autres actifs comprennent la participation dans Schwab, le goodwill, les autres immobilisations incorporelles, les terrains, bâtiments, matériel et mobilier, autres actifs amortissables et actifs au titre de droits d'utilisation, les actifs d'impôt différé, les montants à recevoir des courtiers et des clients et les autres actifs du bilan qui ne sont pas présentés dans les catégories ci-dessus.</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>La réserve pour stabilité intérieure (RSI) a été augmentée pour passer de 3 % à 3,5 % au 1 er novembre 2023. La hausse de 50 pdb reflète le point de vue du BSIF quant aux mesures nécessaires pour améliorer la résilience des plus grandes banques canadiennes. La fourchette de la RSI peut actuellement s'étendre de 0 à 4 %, le niveau effectif étant modifié par le BSIF selon l'évolution du système financier canadien et de l'économie dans son ensemble.</t>
+          <t>5 Les autres actifs comprennent le goodwill, les autres immobilisations incorporelles, les terrains, bâtiments, matériel et mobilier, autres actifs amortissables et actifs au titre de droits d'utilisation, les actifs d'impôt différé, les montants à recevoir des courtiers et des clients et les autres actifs du bilan qui ne sont pas présentés dans les catégories ci-dessus.</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>La réserve pour stabilité intérieure (RSI) a été augmentée pour passer de 3 % à 3,5 % au 1 er novembre 2023 et est demeurée stable depuis. La fourchette de la RSI peut actuellement s'étendre de 0 à 4 %, le niveau effectif étant modifié par le BSIF selon l'évolution du système financier canadien et de l'économie dans son ensemble.</t>
+          <t>Non</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>La réserve pour stabilité intérieure (RSI) a été augmentée de à au novembre et est demeurée stable depuis. Ce changement est substantiel car il reflète une décision stratégique pour renforcer la résilience des grandes banques canadiennes face aux risques systémiques. Cela implique une surveillance accrue des niveaux de capital pour s'assurer que les banques maintiennent cette stabilité dans un contexte économique incertain
-Augmentation de la capacité de résilience des banques face aux chocs économiques</t>
+          <t>La mention de la participation dans Schwab a été supprimée de la liste des autres actifs. Ce changement est substantiel car il indique une modification de la composition des actifs de la banque. Cela implique que la banque doit clarifier la raison de cette suppression et son impact sur le bilan
+La suppression de la participation dans Schwab pourrait indiquer une vente ou une réévaluation de cet actif, affectant potentiellement la structure du bilan</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr"/>
@@ -1200,7 +1304,7 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Gestion des risques</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
@@ -1210,30 +1314,38 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Gestion des risques</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="inlineStr"/>
-      <c r="E18" s="4" t="inlineStr"/>
+          <t>51</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Modification</t>
+        </is>
+      </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>Modification</t>
+          <t>L'approche principale de gestion des activités de financement de la Banque consiste à maximiser l'utilisation des dépôts mobilisés par l'entremise des services bancaires personnels et commerciaux. La réserve de dépôts personnels et commerciaux de la Banque et les comptes de passage de ses activités de gestion de patrimoine et de Schwab (collectivement les dépôts personnels et commerciaux) comptent pour environ 70 % (70 % au 31 octobre 2024) du financement total de la Banque.</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>L'approche principale de gestion des activités de financement de la Banque consiste à maximiser l'utilisation des dépôts mobilisés par l'entremise des services bancaires personnels et commerciaux. La réserve de dépôts personnels et commerciaux de la Banque et les comptes de passage de ses activités de gestion de patrimoine et de Schwab (collectivement les dépôts personnels et commerciaux) comptent pour environ 70 % (70 % au 31 octobre 2024) du financement total de la Banque.</t>
+          <t>L'approche principale de financement de la Banque consiste à maximiser l'utilisation des dépôts mobilisés par l'entremise des services bancaires personnels et commerciaux et de ses activités de gestion de patrimoine, lesquels ont compté pour environ 64 % (63 % au 31 octobre 2024) du financement total de la Banque. Le financement provenant des dépôts non personnels présenté ci-dessous ne tient pas compte des dépôts du secteur Services bancaires de gros de la Banque (y compris ceux du sous-secteur Services bancaires de financement de grandes entreprises et de placement).</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>L'approche principale de financement de la Banque consiste à maximiser l'utilisation des dépôts mobilisés par l'entremise des services bancaires personnels et commerciaux et de ses activités de gestion de patrimoine, lesquels ont compté pour environ 64 % (63 % au 31 octobre 2024) du financement total de la Banque. Le financement provenant des dépôts non personnels présenté ci-dessous ne tient pas compte des dépôts du secteur Services bancaires de gros de la Banque (y compris ceux du sous-secteur Services bancaires de financement de grandes entreprises et de placement).</t>
+          <t>Non</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>Le pourcentage des dépôts personnels et commerciaux a changé, et les dépôts du secteur Services bancaires de gros ont été exclus. Ce changement est substantiel car il modifie la structure de financement de la banque. Cela implique une analyse pour comprendre l'impact de cette exclusion sur la stratégie de financement globale
-La modification de la composition des dépôts pourrait affecter la stabilité et le coût du financement de la banque</t>
+          <t>L'approche de financement de la banque a été modifiée pour inclure les activités de gestion de patrimoine et exclure certains dépôts. Ce changement est substantiel car il modifie la structure de financement de la banque. Cela implique que la banque doit évaluer l'impact de ces changements sur sa stratégie de financement globale
+La modification de l'approche de financement pourrait affecter la stabilité et la flexibilité financière de la banque</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr"/>
@@ -1241,36 +1353,48 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Gestion des risques</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Évolution future des fonds propres réglementaires</t>
+          <t>Actifs liquides</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Gestion du capital</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="inlineStr"/>
-      <c r="E19" s="4" t="inlineStr"/>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Modification</t>
+        </is>
+      </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>Suppression</t>
+          <t>Le total des actifs liquides non grevés a augmenté légèrement de 7 milliards de dollars par rapport à celui au 31 octobre 2024, principalement en raison du produit tiré du financement de gros et des activités connexes liées aux produits.</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>La Banque offre un plan de réinvestissement des dividendes à ses actionnaires ordinaires. La participation à ce plan est facultative et, en vertu des conditions du plan, les dividendes en espèces sur les actions ordinaires servent à acheter des actions ordinaires additionnelles. Au gré de la Banque, les actions ordinaires peuvent être émises sur le capital autorisé, au cours moyen des cinq derniers jours de négociation précédant la date de versement des dividendes, moins un escompte variant entre 0 % et 5 %, au gré de la Banque, ou achetées sur le marché libre, au cours du marché.</t>
-        </is>
-      </c>
-      <c r="H19" s="4" t="inlineStr"/>
+          <t>Le total des actifs liquides non grevés a augmenté de 17 milliards de dollars par rapport à celui au 31 octobre 2024, principalement en raison du produit tiré de la vente de la participation en actions dans Schwab.</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>Le paragraphe sur le plan de réinvestissement des dividendes a été supprimé. Ce changement est substantiel car il affecte les options d'investissement des actionnaires et pourrait influencer la perception du marché. Cela nécessite une investigation pour comprendre les raisons de cette suppression et son impact potentiel sur les actionnaires
-Modification des options d'investissement pour les actionnaires</t>
+          <t>L'augmentation des actifs liquides non grevés a été attribuée à la vente de la participation en actions dans Schwab. Ce changement est substantiel car il modifie la source principale de liquidité de la banque. Cela implique que la banque doit évaluer l'impact de cette vente sur sa stratégie de liquidité à long terme
+La vente de la participation en actions dans Schwab a amélioré la liquidité, mais pourrait réduire les revenus futurs</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr"/>
@@ -1278,7 +1402,7 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Gestion des risques</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
@@ -1288,30 +1412,38 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Gestion des risques</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="inlineStr"/>
-      <c r="E20" s="4" t="inlineStr"/>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>Modification</t>
+        </is>
+      </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>Modification</t>
+          <t>La moyenne des HQLA de la Banque pour le trimestre clos le 31 janvier 2025 a été de 382 milliards de dollars (361 milliards de dollars pour le trimestre clos 31 octobre 2024), les actifs du niveau 1 représentant 86 % (86 % pour le trimestre clos le 31 octobre 2024).</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>Le total des actifs liquides non grevés a augmenté légèrement de 7 milliards de dollars par rapport à celui au 31 octobre 2024, principalement en raison du produit tiré du financement de gros et des activités connexes liées aux produits.</t>
+          <t>La moyenne des HQLA de la Banque pour le trimestre clos le 30 avril 2025 a été de 383 milliards de dollars (382 milliards de dollars pour le trimestre clos le 31 janvier 2025), les actifs du niveau 1 représentant 86 % (86 % pour le trimestre clos le 31 janvier 2025).</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>Le total des actifs liquides non grevés a augmenté de 17 milliards de dollars par rapport à celui au 31 octobre 2024, principalement en raison du produit tiré de la vente de la participation en actions dans Schwab.</t>
+          <t>Non</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>L'augmentation des actifs liquides non grevés a été réévaluée avec une nouvelle raison principale liée à la vente de la participation en actions dans Schwab. Ce changement est substantiel car il modifie la source de liquidité de la banque. Cela implique une vérification de l'impact de cette vente sur la liquidité globale et la stratégie de financement de la banque
-La vente de la participation en Schwab a significativement amélioré la liquidité, ce qui pourrait influencer les décisions futures de financement</t>
+          <t>Les montants des actifs liquides de haute qualité (HQLA) ont été mis à jour pour le trimestre. Ce changement est substantiel car il affecte le calcul des ratios de liquidité réglementaires. Cela implique que la banque doit confirmer ces chiffres pour s'assurer qu'ils sont conformes aux des exigences prudentielles
+Les nouvelles valeurs des HQLA influencent directement la capacité de la banque à répondre aux exigences de liquidité en période de stress</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr"/>
@@ -1319,7 +1451,7 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Gestion des risques</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
@@ -1329,24 +1461,32 @@
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Gestion des risques</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="inlineStr"/>
-      <c r="E21" s="5" t="inlineStr"/>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Modification</t>
+        </is>
+      </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>Modification</t>
+          <t>Le graphique ci-après présente, à une date particulière, l'utilisation de la VaR quotidienne et les produits de négociation nets, présentés en équivalence fiscale, dans le secteur Services bancaires de gros. Les produits de négociation nets comprennent les produits de négociation et les produits d'intérêts nets liés aux positions des portefeuilles de négociation de la Banque utilisés pour la gestion des fonds propres exposés au risque de marché. Le premier trimestre clos le 31 janvier 2025 a compté 4 jours de pertes de négociation et les produits de négociation nets ont été positifs pendant 94 % des jours de Bourse, ce qui reflète une activité de négociation normale. Au cours du trimestre, les pertes pour un jour de Bourse donné n'ont jamais dépassé la VaR.</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>Le graphique ci-après présente, à une date particulière, l'utilisation de la VaR quotidienne et les produits de négociation nets, présentés en équivalence fiscale, dans le secteur Services bancaires de gros. Les produits de négociation nets comprennent les produits de négociation et les produits d'intérêts nets liés aux positions des portefeuilles de négociation de la Banque utilisés pour la gestion des fonds propres exposés au risque de marché. Le premier trimestre clos le 31 janvier 2025 a compté 4 jours de pertes de négociation et les produits de négociation nets ont été positifs pendant 94 % des jours de Bourse, ce qui reflète une activité de négociation normale. Au cours du trimestre, les pertes pour un jour de Bourse donné n'ont jamais dépassé la VaR.</t>
+          <t>Le graphique ci-après présente, à une date particulière, l'utilisation de la VaR quotidienne et les produits de négociation nets, présentés en équivalence fiscale, dans le secteur Services bancaires de gros. Les produits de négociation nets comprennent les produits de négociation et les produits d'intérêts nets liés aux positions des portefeuilles de négociation de la Banque utilisés pour la gestion des fonds propres exposés au risque de marché. Le deuxième trimestre clos le 30 avril 2025 a compté 7 jours de pertes de négociation et les produits de négociation nets ont été positifs pendant 89 % des jours de Bourse, ce qui reflète une activité de négociation normale. Au cours du trimestre, les pertes pour un jour de Bourse donné n'ont jamais dépassé la VaR.</t>
         </is>
       </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>Le graphique ci-après présente, à une date particulière, l'utilisation de la VaR quotidienne et les produits de négociation nets, présentés en équivalence fiscale, dans le secteur Services bancaires de gros. Les produits de négociation nets comprennent les produits de négociation et les produits d'intérêts nets liés aux positions des portefeuilles de négociation de la Banque utilisés pour la gestion des fonds propres exposés au risque de marché. Le deuxième trimestre clos le 30 avril 2025 a compté 7 jours de pertes de négociation et les produits de négociation nets ont été positifs pendant 89 % des jours de Bourse, ce qui reflète une activité de négociation normale. Au cours du trimestre, les pertes pour un jour de Bourse donné n'ont jamais dépassé la VaR.</t>
+          <t>Non</t>
         </is>
       </c>
       <c r="I21" s="5" t="inlineStr"/>
@@ -1355,7 +1495,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Gestion des risques</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
@@ -1365,61 +1505,77 @@
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Gestion des risques</t>
-        </is>
-      </c>
-      <c r="D22" s="5" t="inlineStr"/>
-      <c r="E22" s="5" t="inlineStr"/>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>Modification</t>
+        </is>
+      </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>Modification</t>
+          <t>Le tableau qui suit présente le calcul de la VaR de la TD à la date de clôture du trimestre, la moyenne de la période et les extrêmes (haut et bas).</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
-        <is>
-          <t>Le tableau qui suit présente le calcul de la VaR de la TD à la date de clôture du trimestre, la moyenne de la période et les extrêmes (haut et bas).</t>
-        </is>
-      </c>
-      <c r="H22" s="5" t="inlineStr">
         <is>
           <t>Le tableau qui suit présente le calcul de la VaR de la TD à la date de clôture du trimestre, la moyenne de la période et les extrêmes (haut et bas).
 Négligeable. Il n'est pas important de calculer un effet de diversification, du fait que le haut et le bas peuvent survenir à différents jours pour différents types de risque.</t>
         </is>
       </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
       <c r="I22" s="5" t="inlineStr"/>
       <c r="J22" s="5" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Gestion des risques</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Exigences en matière de fonds propres du BSIF en vertu de Bâle III</t>
+          <t>Risque de taux d'intérêt (autre que de négociation) structurel</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Gestion du capital</t>
-        </is>
-      </c>
-      <c r="D23" s="5" t="inlineStr"/>
-      <c r="E23" s="5" t="inlineStr"/>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Modification</t>
+        </is>
+      </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>Modification</t>
+          <t>Le tableau suivant présente l'incidence potentielle avant impôt d'une augmentation ou diminution immédiate et soutenue de 100 pdb des taux d'intérêt sur les mesures de la sensibilité de la valeur économique des capitaux propres attribuables aux actionnaires et de la sensibilité des produits d'intérêts nets.</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>Le 1 er novembre 2023, la Banque a mis en œuvre le Cadre de capacité totale d'absorption des pertes par établissement des sociétés mères de banques d'importance systémique intérieure du BSIF. Ce cadre, qui établit une mesure fondée sur le risque, veille à ce qu'une BISI non viable dispose d'une capacité d'absorption des pertes suffisante par établissement (entité juridique distincte) afin d'assurer sa résolution. La Banque respecte les exigences énoncées dans ce cadre.</t>
+          <t>Le tableau suivant présente l'incidence potentielle avant impôt d'une augmentation ou diminution immédiate et soutenue de 100 pdb des taux d'intérêt sur les mesures de la sensibilité de la valeur économique des capitaux propres attribuables aux actionnaires et de la sensibilité des produits d'intérêts nets.</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
         <is>
-          <t>La Banque a mis en œuvre le Cadre de capacité totale d'absorption des pertes par établissement des sociétés mères de banques d'importance systémique intérieure du BSIF. Ce cadre, qui établit une mesure fondée sur le risque, veille à ce qu'une BISI non viable dispose d'une capacité d'absorption des pertes suffisante par établissement (entité juridique distincte) afin d'assurer sa résolution. La Banque respecte les exigences énoncées dans ce cadre.</t>
+          <t>Non</t>
         </is>
       </c>
       <c r="I23" s="5" t="inlineStr"/>
@@ -1428,41 +1584,129 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Gestion du capital</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Évolution future des fonds propres réglementaires</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>Gestion du capital</t>
-        </is>
-      </c>
-      <c r="D24" s="5" t="inlineStr"/>
-      <c r="E24" s="5" t="inlineStr"/>
-      <c r="F24" s="5" t="inlineStr">
-        <is>
-          <t>Modification</t>
-        </is>
-      </c>
+          <t>Exigences en matière de fonds propres du BSIF en vertu de Bâle III</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr"/>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>Ajout</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr"/>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>Le 26 février 2025, le conseil d'administration a approuvé un dividende de un dollar et cinq cents (1,05 $) par action ordinaire entièrement libérée du capital social de la Banque pour le trimestre se terminant le 30 avril 2025. Ce dividende sera payable à compter du 30 avril 2025 aux actionnaires inscrits à la fermeture des bureaux le 10 avril 2025.</t>
+          <t>Le tableau ci-après présente des détails sur la situation des fonds propres réglementaires de la Banque.</t>
         </is>
       </c>
       <c r="H24" s="5" t="inlineStr">
         <is>
-          <t>Le 21 mai 2025, le conseil d'administration a approuvé un dividende de un dollar et cinq cents (1,05 $) par action ordinaire entièrement libérée du capital social de la Banque pour le trimestre se terminant le 31 juillet 2025. Ce dividende sera payable à compter du 31 juillet 2025 aux actionnaires inscrits à la fermeture des bureaux le 10 juillet 2025.</t>
+          <t>Non</t>
         </is>
       </c>
       <c r="I24" s="5" t="inlineStr"/>
       <c r="J24" s="5" t="inlineStr"/>
     </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Gestion du capital</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Exigences en matière de fonds propres du BSIF en vertu de Bâle III</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>Modification</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>Le 1 er novembre 2023, la Banque a mis en œuvre le Cadre de capacité totale d'absorption des pertes par établissement des sociétés mères de banques d'importance systémique intérieure du BSIF. Ce cadre, qui établit une mesure fondée sur le risque, veille à ce qu'une BISI non viable dispose d'une capacité d'absorption des pertes suffisante par établissement (entité juridique distincte) afin d'assurer sa résolution. La Banque respecte les exigences énoncées dans ce cadre.</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>La Banque a mis en œuvre le Cadre de capacité totale d'absorption des pertes par établissement des sociétés mères de banques d'importance systémique intérieure du BSIF. Ce cadre, qui établit une mesure fondée sur le risque, veille à ce qu'une BISI non viable dispose d'une capacité d'absorption des pertes suffisante par établissement (entité juridique distincte) afin d'assurer sa résolution. La Banque respecte les exigences énoncées dans ce cadre.</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="I25" s="5" t="inlineStr"/>
+      <c r="J25" s="5" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Gestion du capital</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Évolution future des fonds propres réglementaires</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>Modification</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>Le 26 février 2025, le conseil d'administration a approuvé un dividende de un dollar et cinq cents (1,05 $) par action ordinaire entièrement libérée du capital social de la Banque pour le trimestre se terminant le 30 avril 2025. Ce dividende sera payable à compter du 30 avril 2025 aux actionnaires inscrits à la fermeture des bureaux le 10 avril 2025.</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>Le 21 mai 2025, le conseil d'administration a approuvé un dividende de un dollar et cinq cents (1,05 $) par action ordinaire entièrement libérée du capital social de la Banque pour le trimestre se terminant le 31 juillet 2025. Ce dividende sera payable à compter du 31 juillet 2025 aux actionnaires inscrits à la fermeture des bureaux le 10 juillet 2025.</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="I26" s="5" t="inlineStr"/>
+      <c r="J26" s="5" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J24"/>
+  <autoFilter ref="A1:J26"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>